<commit_message>
Changes updated acc #2
</commit_message>
<xml_diff>
--- a/Documents/Client-Files/BOM/Digikey_BOM.xlsx
+++ b/Documents/Client-Files/BOM/Digikey_BOM.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="145">
   <si>
-    <t>Bill of Material (BOM) for Josh</t>
+    <t>Bill of Material (BOM) for Tim Sefton</t>
   </si>
   <si>
     <t>S. No.</t>
@@ -120,7 +120,7 @@
 </t>
   </si>
   <si>
-    <t>C3-C6</t>
+    <t>C3,C4,C5C6</t>
   </si>
   <si>
     <t>CL21A106KOFNNNE</t>
@@ -136,7 +136,7 @@
 </t>
   </si>
   <si>
-    <t>R1,2</t>
+    <t>R1,R2</t>
   </si>
   <si>
     <t>Res0603</t>
@@ -169,7 +169,7 @@
 </t>
   </si>
   <si>
-    <t>R4,5,7,10,11</t>
+    <t>R4,R5,R7,R10,R11</t>
   </si>
   <si>
     <t>Res0805</t>
@@ -185,7 +185,7 @@
 </t>
   </si>
   <si>
-    <t>R8,9,12,13</t>
+    <t>R8,R9,R12,R13</t>
   </si>
   <si>
     <t>RC0805JR-0710KL</t>
@@ -230,7 +230,7 @@
 </t>
   </si>
   <si>
-    <t>D1:D5</t>
+    <t>D1,D2,D3,D4,D5</t>
   </si>
   <si>
     <t>SOD323F</t>
@@ -268,7 +268,7 @@
 </t>
   </si>
   <si>
-    <t>Q1:Q5</t>
+    <t>Q1,Q2,Q3,Q4,Q5</t>
   </si>
   <si>
     <t xml:space="preserve"> SOT323</t>
@@ -288,7 +288,7 @@
 </t>
   </si>
   <si>
-    <t>K1-K2</t>
+    <t>K1,K2</t>
   </si>
   <si>
     <t>Custom</t>
@@ -310,7 +310,7 @@
     <t>Songle relay</t>
   </si>
   <si>
-    <t>K3-K5</t>
+    <t>K3,K4,K5</t>
   </si>
   <si>
     <t>SLA-05VDC-S-L-C</t>
@@ -386,7 +386,7 @@
 </t>
   </si>
   <si>
-    <t>X8</t>
+    <t>U8</t>
   </si>
   <si>
     <t>ESP32-WROOM-32</t>
@@ -429,7 +429,7 @@
 </t>
   </si>
   <si>
-    <t>x3-x7 , x11 , x12</t>
+    <t>J3,J4,J5,J6,J7, J11 , J12</t>
   </si>
   <si>
     <t>HDR1X3</t>
@@ -449,7 +449,7 @@
 </t>
   </si>
   <si>
-    <t>x1,x2,x9,x10,x13</t>
+    <t>J1,J2,J9,J10,J13</t>
   </si>
   <si>
     <t>HDR1X2</t>
@@ -470,16 +470,16 @@
     <t>Aliexpress</t>
   </si>
   <si>
+    <t>NOTE:</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total Component Cost </t>
   </si>
   <si>
-    <t>NOTE:</t>
+    <t>Songle relay available at hallroad only:</t>
   </si>
   <si>
     <t>Single Board Cost</t>
-  </si>
-  <si>
-    <t>Songle relay available at hallroad only:</t>
   </si>
 </sst>
 </file>
@@ -487,11 +487,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="28">
     <font>
@@ -564,24 +564,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -596,25 +594,34 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -626,8 +633,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -642,29 +664,15 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -678,16 +686,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -733,7 +733,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -745,13 +763,139 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -763,157 +907,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1171,6 +1171,69 @@
       </top>
       <bottom style="medium">
         <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1192,59 +1255,11 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
       <bottom style="double">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1257,35 +1272,20 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1298,131 +1298,131 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="26" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="22" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1492,12 +1492,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1516,9 +1510,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1529,12 +1520,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1552,9 +1537,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1567,9 +1549,6 @@
     <xf numFmtId="8" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1579,9 +1558,6 @@
     <xf numFmtId="8" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1591,9 +1567,6 @@
     <xf numFmtId="8" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1612,40 +1585,19 @@
     <xf numFmtId="8" fontId="3" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="8" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="8" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="8" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1675,28 +1627,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
@@ -2058,12 +1998,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:T30"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col min="1" max="1" width="7.28571428571429" customWidth="1"/>
     <col min="2" max="2" width="14.2857142857143" customWidth="1"/>
     <col min="3" max="3" width="41.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="16.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="22.1428571428571" customWidth="1"/>
     <col min="6" max="6" width="30.7142857142857" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
@@ -2077,6 +2017,8 @@
     <col min="15" max="15" width="22.1428571428571" customWidth="1"/>
     <col min="16" max="16" width="15" customWidth="1"/>
     <col min="17" max="17" width="31" customWidth="1"/>
+    <col min="18" max="133" width="9.14285714285714" hidden="1" customWidth="1"/>
+    <col min="134" max="16384" width="9.14285714285714" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="16.5" spans="1:18">
@@ -2099,7 +2041,7 @@
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
-      <c r="R1" s="79"/>
+      <c r="R1" s="63"/>
     </row>
     <row r="2" ht="16.5" spans="1:18">
       <c r="A2" s="2" t="s">
@@ -2153,7 +2095,7 @@
       <c r="Q2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="79"/>
+      <c r="R2" s="63"/>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" s="5">
@@ -2168,7 +2110,7 @@
       <c r="D3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="92" t="s">
+      <c r="E3" s="72" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -2186,31 +2128,31 @@
       <c r="J3" s="10">
         <v>1</v>
       </c>
-      <c r="K3" s="43">
+      <c r="K3" s="8">
         <f>J3*5</f>
         <v>5</v>
       </c>
-      <c r="L3" s="44" t="s">
+      <c r="L3" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="M3" s="45">
+      <c r="M3" s="39">
         <v>0.1</v>
       </c>
-      <c r="N3" s="46">
+      <c r="N3" s="40">
         <f>M3*J3</f>
         <v>0.1</v>
       </c>
-      <c r="O3" s="47">
+      <c r="O3" s="41">
         <v>0.1</v>
       </c>
-      <c r="P3" s="46">
+      <c r="P3" s="40">
         <f>O3*K3</f>
         <v>0.5</v>
       </c>
-      <c r="Q3" s="80"/>
-      <c r="R3" s="81"/>
-      <c r="S3" s="39"/>
-      <c r="T3" s="39"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="65"/>
+      <c r="S3" s="34"/>
+      <c r="T3" s="34"/>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" s="5">
@@ -2224,7 +2166,7 @@
       <c r="D4" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="93" t="s">
+      <c r="E4" s="73" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="13" t="s">
@@ -2233,7 +2175,7 @@
       <c r="G4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="94" t="s">
+      <c r="H4" s="74" t="s">
         <v>30</v>
       </c>
       <c r="I4" s="15" t="s">
@@ -2242,33 +2184,33 @@
       <c r="J4" s="15">
         <v>1</v>
       </c>
-      <c r="K4" s="48">
+      <c r="K4" s="13">
         <f t="shared" ref="K4:K23" si="0">J4*5</f>
         <v>5</v>
       </c>
-      <c r="L4" s="49" t="s">
+      <c r="L4" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="50">
+      <c r="M4" s="43">
         <v>0.1</v>
       </c>
-      <c r="N4" s="51">
+      <c r="N4" s="44">
         <f t="shared" ref="N4:N24" si="1">M4*J4</f>
         <v>0.1</v>
       </c>
-      <c r="O4" s="51">
+      <c r="O4" s="44">
         <v>0.1</v>
       </c>
-      <c r="P4" s="51">
+      <c r="P4" s="44">
         <f t="shared" ref="P4:P23" si="2">O4*K4</f>
         <v>0.5</v>
       </c>
-      <c r="Q4" s="82"/>
-      <c r="R4" s="81"/>
-      <c r="S4" s="39"/>
-      <c r="T4" s="39"/>
+      <c r="Q4" s="66"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="34"/>
+      <c r="T4" s="34"/>
     </row>
-    <row r="5" ht="15.75" spans="1:20">
+    <row r="5" spans="1:20">
       <c r="A5" s="5">
         <f t="shared" ref="A5:A24" si="3">A4+1</f>
         <v>3</v>
@@ -2280,7 +2222,7 @@
       <c r="D5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="95" t="s">
+      <c r="E5" s="75" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="18" t="s">
@@ -2289,7 +2231,7 @@
       <c r="G5" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="96" t="s">
+      <c r="H5" s="76" t="s">
         <v>30</v>
       </c>
       <c r="I5" s="20" t="s">
@@ -2298,31 +2240,31 @@
       <c r="J5" s="20">
         <v>4</v>
       </c>
-      <c r="K5" s="52">
+      <c r="K5" s="18">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L5" s="53" t="s">
+      <c r="L5" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M5" s="54">
+      <c r="M5" s="46">
         <v>0.17</v>
       </c>
-      <c r="N5" s="55">
+      <c r="N5" s="47">
         <f t="shared" si="1"/>
         <v>0.68</v>
       </c>
-      <c r="O5" s="55">
+      <c r="O5" s="47">
         <v>0.12</v>
       </c>
-      <c r="P5" s="55">
+      <c r="P5" s="47">
         <f t="shared" si="2"/>
         <v>2.4</v>
       </c>
-      <c r="Q5" s="83"/>
-      <c r="R5" s="81"/>
-      <c r="S5" s="39"/>
-      <c r="T5" s="39"/>
+      <c r="Q5" s="67"/>
+      <c r="R5" s="65"/>
+      <c r="S5" s="34"/>
+      <c r="T5" s="34"/>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" s="5">
@@ -2347,7 +2289,7 @@
       <c r="G6" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="97" t="s">
+      <c r="H6" s="77" t="s">
         <v>30</v>
       </c>
       <c r="I6" s="10" t="s">
@@ -2356,31 +2298,31 @@
       <c r="J6" s="10">
         <v>2</v>
       </c>
-      <c r="K6" s="43">
+      <c r="K6" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L6" s="44" t="s">
+      <c r="L6" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="M6" s="45">
+      <c r="M6" s="39">
         <v>0.1</v>
       </c>
-      <c r="N6" s="46">
+      <c r="N6" s="40">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="O6" s="46">
+      <c r="O6" s="40">
         <v>0.02</v>
       </c>
-      <c r="P6" s="46">
+      <c r="P6" s="40">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
-      <c r="Q6" s="80"/>
-      <c r="R6" s="81"/>
-      <c r="S6" s="39"/>
-      <c r="T6" s="39"/>
+      <c r="Q6" s="64"/>
+      <c r="R6" s="65"/>
+      <c r="S6" s="34"/>
+      <c r="T6" s="34"/>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" s="5">
@@ -2403,7 +2345,7 @@
       <c r="G7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="94" t="s">
+      <c r="H7" s="74" t="s">
         <v>30</v>
       </c>
       <c r="I7" s="15" t="s">
@@ -2412,31 +2354,31 @@
       <c r="J7" s="15">
         <v>1</v>
       </c>
-      <c r="K7" s="48">
+      <c r="K7" s="13">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L7" s="49" t="s">
+      <c r="L7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="M7" s="50">
+      <c r="M7" s="43">
         <v>0.1</v>
       </c>
-      <c r="N7" s="51">
+      <c r="N7" s="44">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O7" s="51">
+      <c r="O7" s="44">
         <v>0.02</v>
       </c>
-      <c r="P7" s="51">
+      <c r="P7" s="44">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="Q7" s="82"/>
-      <c r="R7" s="81"/>
-      <c r="S7" s="39"/>
-      <c r="T7" s="39"/>
+      <c r="Q7" s="66"/>
+      <c r="R7" s="65"/>
+      <c r="S7" s="34"/>
+      <c r="T7" s="34"/>
     </row>
     <row r="8" spans="1:20">
       <c r="A8" s="5">
@@ -2459,7 +2401,7 @@
       <c r="G8" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="H8" s="94" t="s">
+      <c r="H8" s="74" t="s">
         <v>30</v>
       </c>
       <c r="I8" s="15" t="s">
@@ -2468,31 +2410,31 @@
       <c r="J8" s="15">
         <v>5</v>
       </c>
-      <c r="K8" s="48">
+      <c r="K8" s="13">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L8" s="49" t="s">
+      <c r="L8" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="M8" s="50">
+      <c r="M8" s="43">
         <v>0.1</v>
       </c>
-      <c r="N8" s="51">
+      <c r="N8" s="44">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="O8" s="51">
+      <c r="O8" s="44">
         <v>0.036</v>
       </c>
-      <c r="P8" s="51">
+      <c r="P8" s="44">
         <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
-      <c r="Q8" s="82"/>
-      <c r="R8" s="81"/>
-      <c r="S8" s="39"/>
-      <c r="T8" s="39"/>
+      <c r="Q8" s="66"/>
+      <c r="R8" s="65"/>
+      <c r="S8" s="34"/>
+      <c r="T8" s="34"/>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" s="5">
@@ -2515,7 +2457,7 @@
       <c r="G9" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="94" t="s">
+      <c r="H9" s="74" t="s">
         <v>30</v>
       </c>
       <c r="I9" s="15" t="s">
@@ -2524,31 +2466,31 @@
       <c r="J9" s="15">
         <v>4</v>
       </c>
-      <c r="K9" s="48">
+      <c r="K9" s="13">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L9" s="49" t="s">
+      <c r="L9" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="M9" s="50">
+      <c r="M9" s="43">
         <v>0.1</v>
       </c>
-      <c r="N9" s="51">
+      <c r="N9" s="44">
         <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
-      <c r="O9" s="51">
+      <c r="O9" s="44">
         <v>0.036</v>
       </c>
-      <c r="P9" s="51">
+      <c r="P9" s="44">
         <f t="shared" si="2"/>
         <v>0.72</v>
       </c>
-      <c r="Q9" s="82"/>
-      <c r="R9" s="81"/>
-      <c r="S9" s="39"/>
-      <c r="T9" s="39"/>
+      <c r="Q9" s="66"/>
+      <c r="R9" s="65"/>
+      <c r="S9" s="34"/>
+      <c r="T9" s="34"/>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="5">
@@ -2571,7 +2513,7 @@
       <c r="G10" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="H10" s="94" t="s">
+      <c r="H10" s="74" t="s">
         <v>30</v>
       </c>
       <c r="I10" s="15" t="s">
@@ -2580,31 +2522,31 @@
       <c r="J10" s="15">
         <v>1</v>
       </c>
-      <c r="K10" s="48">
+      <c r="K10" s="13">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L10" s="49" t="s">
+      <c r="L10" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="M10" s="50">
+      <c r="M10" s="43">
         <v>0.1</v>
       </c>
-      <c r="N10" s="51">
+      <c r="N10" s="44">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O10" s="51">
+      <c r="O10" s="44">
         <v>0.1</v>
       </c>
-      <c r="P10" s="51">
+      <c r="P10" s="44">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q10" s="82"/>
-      <c r="R10" s="81"/>
-      <c r="S10" s="39"/>
-      <c r="T10" s="39"/>
+      <c r="Q10" s="66"/>
+      <c r="R10" s="65"/>
+      <c r="S10" s="34"/>
+      <c r="T10" s="34"/>
     </row>
     <row r="11" ht="15.75" spans="1:20">
       <c r="A11" s="5">
@@ -2636,38 +2578,38 @@
       <c r="J11" s="20">
         <v>1</v>
       </c>
-      <c r="K11" s="52">
+      <c r="K11" s="18">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L11" s="53" t="s">
+      <c r="L11" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M11" s="54">
+      <c r="M11" s="46">
         <v>0.66</v>
       </c>
-      <c r="N11" s="55">
+      <c r="N11" s="47">
         <f t="shared" si="1"/>
         <v>0.66</v>
       </c>
-      <c r="O11" s="55">
+      <c r="O11" s="47">
         <v>0.66</v>
       </c>
-      <c r="P11" s="55">
+      <c r="P11" s="47">
         <f t="shared" si="2"/>
         <v>3.3</v>
       </c>
-      <c r="Q11" s="83"/>
-      <c r="R11" s="81"/>
-      <c r="S11" s="39"/>
-      <c r="T11" s="39"/>
+      <c r="Q11" s="67"/>
+      <c r="R11" s="65"/>
+      <c r="S11" s="34"/>
+      <c r="T11" s="34"/>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" s="5">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="6" t="s">
         <v>65</v>
       </c>
       <c r="C12" s="21" t="s">
@@ -2685,47 +2627,47 @@
       <c r="G12" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="97" t="s">
-        <v>30</v>
-      </c>
-      <c r="I12" s="97" t="s">
+      <c r="H12" s="77" t="s">
+        <v>30</v>
+      </c>
+      <c r="I12" s="77" t="s">
         <v>30</v>
       </c>
       <c r="J12" s="10">
         <v>5</v>
       </c>
-      <c r="K12" s="43">
+      <c r="K12" s="8">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L12" s="44" t="s">
+      <c r="L12" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="M12" s="45">
+      <c r="M12" s="39">
         <v>0.21</v>
       </c>
-      <c r="N12" s="46">
+      <c r="N12" s="40">
         <f t="shared" si="1"/>
         <v>1.05</v>
       </c>
-      <c r="O12" s="46">
+      <c r="O12" s="40">
         <v>0.192</v>
       </c>
-      <c r="P12" s="46">
+      <c r="P12" s="40">
         <f t="shared" si="2"/>
         <v>4.8</v>
       </c>
-      <c r="Q12" s="80"/>
-      <c r="R12" s="81"/>
-      <c r="S12" s="39"/>
-      <c r="T12" s="39"/>
+      <c r="Q12" s="64"/>
+      <c r="R12" s="65"/>
+      <c r="S12" s="34"/>
+      <c r="T12" s="34"/>
     </row>
     <row r="13" ht="15.75" spans="1:20">
       <c r="A13" s="5">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
-      <c r="B13" s="24"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="17" t="s">
         <v>71</v>
       </c>
@@ -2744,97 +2686,97 @@
       <c r="H13" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="I13" s="96" t="s">
+      <c r="I13" s="76" t="s">
         <v>30</v>
       </c>
       <c r="J13" s="20">
         <v>1</v>
       </c>
-      <c r="K13" s="52">
+      <c r="K13" s="18">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L13" s="53" t="s">
+      <c r="L13" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M13" s="54">
+      <c r="M13" s="46">
         <v>0.42</v>
       </c>
-      <c r="N13" s="55">
+      <c r="N13" s="47">
         <f t="shared" si="1"/>
         <v>0.42</v>
       </c>
-      <c r="O13" s="55">
+      <c r="O13" s="47">
         <v>0.42</v>
       </c>
-      <c r="P13" s="55">
+      <c r="P13" s="47">
         <f t="shared" si="2"/>
         <v>2.1</v>
       </c>
-      <c r="Q13" s="84" t="s">
+      <c r="Q13" s="67" t="s">
         <v>76</v>
       </c>
-      <c r="R13" s="85"/>
-      <c r="S13" s="39"/>
-      <c r="T13" s="39"/>
+      <c r="R13" s="68"/>
+      <c r="S13" s="34"/>
+      <c r="T13" s="34"/>
     </row>
-    <row r="14" ht="15.75" spans="1:20">
+    <row r="14" spans="1:20">
       <c r="A14" s="5">
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="F14" s="27" t="s">
+      <c r="F14" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="G14" s="28" t="s">
+      <c r="G14" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="I14" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="J14" s="28">
+      <c r="H14" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="I14" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="J14" s="26">
         <v>5</v>
       </c>
-      <c r="K14" s="56">
+      <c r="K14" s="25">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L14" s="57" t="s">
+      <c r="L14" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="M14" s="58">
+      <c r="M14" s="49">
         <v>0.2</v>
       </c>
-      <c r="N14" s="59">
+      <c r="N14" s="50">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="O14" s="59">
+      <c r="O14" s="50">
         <v>0.182</v>
       </c>
-      <c r="P14" s="59">
+      <c r="P14" s="50">
         <f t="shared" si="2"/>
         <v>4.55</v>
       </c>
-      <c r="Q14" s="86"/>
-      <c r="R14" s="85"/>
-      <c r="S14" s="39"/>
-      <c r="T14" s="39"/>
+      <c r="Q14" s="69"/>
+      <c r="R14" s="68"/>
+      <c r="S14" s="34"/>
+      <c r="T14" s="34"/>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" s="5">
@@ -2862,143 +2804,143 @@
       <c r="H15" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="I15" s="97" t="s">
+      <c r="I15" s="77" t="s">
         <v>30</v>
       </c>
       <c r="J15" s="10">
         <v>2</v>
       </c>
-      <c r="K15" s="43">
+      <c r="K15" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L15" s="44" t="s">
+      <c r="L15" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="M15" s="45">
+      <c r="M15" s="39">
         <v>1.18</v>
       </c>
-      <c r="N15" s="46">
+      <c r="N15" s="40">
         <f t="shared" si="1"/>
         <v>2.36</v>
       </c>
-      <c r="O15" s="46">
+      <c r="O15" s="40">
         <v>1.11</v>
       </c>
-      <c r="P15" s="46">
+      <c r="P15" s="40">
         <f t="shared" si="2"/>
         <v>11.1</v>
       </c>
-      <c r="Q15" s="87" t="s">
+      <c r="Q15" s="64" t="s">
         <v>90</v>
       </c>
-      <c r="R15" s="85"/>
-      <c r="S15" s="39"/>
-      <c r="T15" s="39"/>
+      <c r="R15" s="68"/>
+      <c r="S15" s="34"/>
+      <c r="T15" s="34"/>
     </row>
-    <row r="16" ht="15.75" spans="1:20">
+    <row r="16" spans="1:20">
       <c r="A16" s="5">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="B16" s="16"/>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="D16" s="30" t="s">
+      <c r="D16" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="E16" s="31"/>
-      <c r="F16" s="30" t="s">
+      <c r="E16" s="28"/>
+      <c r="F16" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="G16" s="32"/>
-      <c r="H16" s="99" t="s">
-        <v>30</v>
-      </c>
-      <c r="I16" s="99" t="s">
-        <v>30</v>
-      </c>
-      <c r="J16" s="32">
+      <c r="G16" s="29"/>
+      <c r="H16" s="79" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16" s="79" t="s">
+        <v>30</v>
+      </c>
+      <c r="J16" s="29">
         <v>3</v>
       </c>
-      <c r="K16" s="31">
+      <c r="K16" s="28">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="L16" s="60"/>
-      <c r="M16" s="61"/>
-      <c r="N16" s="62">
+      <c r="L16" s="51"/>
+      <c r="M16" s="52"/>
+      <c r="N16" s="53">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O16" s="62"/>
-      <c r="P16" s="62">
+      <c r="O16" s="53"/>
+      <c r="P16" s="53">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="Q16" s="88"/>
-      <c r="R16" s="85"/>
-      <c r="S16" s="39"/>
-      <c r="T16" s="39"/>
+      <c r="Q16" s="70"/>
+      <c r="R16" s="68"/>
+      <c r="S16" s="34"/>
+      <c r="T16" s="34"/>
     </row>
     <row r="17" ht="15.75" spans="1:20">
       <c r="A17" s="5">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="G17" s="28" t="s">
+      <c r="G17" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="H17" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="I17" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="J17" s="28">
+      <c r="H17" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="I17" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="J17" s="26">
         <v>2</v>
       </c>
-      <c r="K17" s="56">
+      <c r="K17" s="25">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L17" s="57" t="s">
+      <c r="L17" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="M17" s="58">
+      <c r="M17" s="49">
         <v>0.57</v>
       </c>
-      <c r="N17" s="59">
+      <c r="N17" s="50">
         <f t="shared" si="1"/>
         <v>1.14</v>
       </c>
-      <c r="O17" s="59">
+      <c r="O17" s="50">
         <v>0.546</v>
       </c>
-      <c r="P17" s="59">
+      <c r="P17" s="50">
         <f t="shared" si="2"/>
         <v>5.46</v>
       </c>
-      <c r="Q17" s="86"/>
-      <c r="R17" s="85"/>
-      <c r="S17" s="39"/>
-      <c r="T17" s="39"/>
+      <c r="Q17" s="69"/>
+      <c r="R17" s="68"/>
+      <c r="S17" s="34"/>
+      <c r="T17" s="34"/>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" s="5">
@@ -3020,45 +2962,45 @@
       <c r="F18" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="G18" s="33" t="s">
+      <c r="G18" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="H18" s="33" t="s">
+      <c r="H18" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="I18" s="100" t="s">
-        <v>30</v>
-      </c>
-      <c r="J18" s="33">
+      <c r="I18" s="80" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" s="30">
         <v>1</v>
       </c>
-      <c r="K18" s="63">
+      <c r="K18" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L18" s="44" t="s">
+      <c r="L18" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="M18" s="64">
+      <c r="M18" s="54">
         <v>0.5</v>
       </c>
-      <c r="N18" s="65">
+      <c r="N18" s="40">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="O18" s="65">
+      <c r="O18" s="40">
         <v>0.5</v>
       </c>
-      <c r="P18" s="65">
+      <c r="P18" s="40">
         <f t="shared" si="2"/>
         <v>2.5</v>
       </c>
-      <c r="Q18" s="87" t="s">
+      <c r="Q18" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="R18" s="85"/>
-      <c r="S18" s="39"/>
-      <c r="T18" s="39"/>
+      <c r="R18" s="68"/>
+      <c r="S18" s="34"/>
+      <c r="T18" s="34"/>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" s="5">
@@ -3078,47 +3020,47 @@
       <c r="F19" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="H19" s="34" t="s">
+      <c r="H19" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="I19" s="101" t="s">
-        <v>30</v>
-      </c>
-      <c r="J19" s="34">
+      <c r="I19" s="81" t="s">
+        <v>30</v>
+      </c>
+      <c r="J19" s="31">
         <v>1</v>
       </c>
-      <c r="K19" s="66">
+      <c r="K19" s="13">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L19" s="49" t="s">
+      <c r="L19" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="M19" s="67">
+      <c r="M19" s="55">
         <v>0.99</v>
       </c>
-      <c r="N19" s="68">
+      <c r="N19" s="44">
         <f t="shared" si="1"/>
         <v>0.99</v>
       </c>
-      <c r="O19" s="68">
+      <c r="O19" s="44">
         <v>0.99</v>
       </c>
-      <c r="P19" s="68">
+      <c r="P19" s="44">
         <f t="shared" si="2"/>
         <v>4.95</v>
       </c>
-      <c r="Q19" s="89" t="s">
+      <c r="Q19" s="66" t="s">
         <v>113</v>
       </c>
-      <c r="R19" s="85"/>
-      <c r="S19" s="39"/>
-      <c r="T19" s="39"/>
+      <c r="R19" s="68"/>
+      <c r="S19" s="34"/>
+      <c r="T19" s="34"/>
     </row>
-    <row r="20" ht="15.75" spans="1:20">
+    <row r="20" spans="1:20">
       <c r="A20" s="5">
         <f t="shared" si="3"/>
         <v>18</v>
@@ -3136,45 +3078,45 @@
       <c r="F20" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="G20" s="35" t="s">
+      <c r="G20" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="H20" s="35" t="s">
+      <c r="H20" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="I20" s="102" t="s">
-        <v>30</v>
-      </c>
-      <c r="J20" s="35">
+      <c r="I20" s="82" t="s">
+        <v>30</v>
+      </c>
+      <c r="J20" s="32">
         <v>1</v>
       </c>
-      <c r="K20" s="69">
+      <c r="K20" s="18">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L20" s="53" t="s">
+      <c r="L20" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="M20" s="70">
+      <c r="M20" s="56">
         <v>3</v>
       </c>
-      <c r="N20" s="71">
+      <c r="N20" s="47">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="O20" s="71">
+      <c r="O20" s="47">
         <v>3</v>
       </c>
-      <c r="P20" s="71">
+      <c r="P20" s="47">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="Q20" s="84" t="s">
+      <c r="Q20" s="67" t="s">
         <v>120</v>
       </c>
-      <c r="R20" s="85"/>
-      <c r="S20" s="39"/>
-      <c r="T20" s="39"/>
+      <c r="R20" s="68"/>
+      <c r="S20" s="34"/>
+      <c r="T20" s="34"/>
     </row>
     <row r="21" spans="1:20">
       <c r="A21" s="5">
@@ -3199,40 +3141,40 @@
       <c r="G21" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="H21" s="97" t="s">
-        <v>30</v>
-      </c>
-      <c r="I21" s="97" t="s">
+      <c r="H21" s="77" t="s">
+        <v>30</v>
+      </c>
+      <c r="I21" s="77" t="s">
         <v>30</v>
       </c>
       <c r="J21" s="10">
         <v>1</v>
       </c>
-      <c r="K21" s="43">
+      <c r="K21" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L21" s="72" t="s">
+      <c r="L21" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="M21" s="45">
+      <c r="M21" s="39">
         <v>0.28</v>
       </c>
-      <c r="N21" s="46">
+      <c r="N21" s="40">
         <f t="shared" si="1"/>
         <v>0.28</v>
       </c>
-      <c r="O21" s="46">
+      <c r="O21" s="40">
         <v>0.28</v>
       </c>
-      <c r="P21" s="46">
+      <c r="P21" s="40">
         <f t="shared" si="2"/>
         <v>1.4</v>
       </c>
-      <c r="Q21" s="80"/>
-      <c r="R21" s="85"/>
-      <c r="S21" s="39"/>
-      <c r="T21" s="39"/>
+      <c r="Q21" s="64"/>
+      <c r="R21" s="68"/>
+      <c r="S21" s="34"/>
+      <c r="T21" s="34"/>
     </row>
     <row r="22" spans="1:20">
       <c r="A22" s="5">
@@ -3255,44 +3197,44 @@
       <c r="G22" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="H22" s="94" t="s">
-        <v>30</v>
-      </c>
-      <c r="I22" s="94" t="s">
+      <c r="H22" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22" s="74" t="s">
         <v>30</v>
       </c>
       <c r="J22" s="15">
         <v>7</v>
       </c>
-      <c r="K22" s="48">
+      <c r="K22" s="13">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="L22" s="73" t="s">
+      <c r="L22" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="M22" s="50">
+      <c r="M22" s="43">
         <v>3.52</v>
       </c>
-      <c r="N22" s="51">
+      <c r="N22" s="44">
         <f t="shared" si="1"/>
         <v>24.64</v>
       </c>
-      <c r="O22" s="51">
+      <c r="O22" s="44">
         <v>3.424</v>
       </c>
-      <c r="P22" s="51">
+      <c r="P22" s="44">
         <f t="shared" si="2"/>
         <v>119.84</v>
       </c>
-      <c r="Q22" s="89" t="s">
+      <c r="Q22" s="66" t="s">
         <v>132</v>
       </c>
-      <c r="R22" s="85"/>
-      <c r="S22" s="39"/>
-      <c r="T22" s="39"/>
+      <c r="R22" s="68"/>
+      <c r="S22" s="34"/>
+      <c r="T22" s="34"/>
     </row>
-    <row r="23" ht="15.75" spans="1:20">
+    <row r="23" spans="1:20">
       <c r="A23" s="5">
         <f t="shared" si="3"/>
         <v>21</v>
@@ -3313,157 +3255,154 @@
       <c r="G23" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="H23" s="96" t="s">
-        <v>30</v>
-      </c>
-      <c r="I23" s="96" t="s">
+      <c r="H23" s="76" t="s">
+        <v>30</v>
+      </c>
+      <c r="I23" s="76" t="s">
         <v>30</v>
       </c>
       <c r="J23" s="20">
         <v>5</v>
       </c>
-      <c r="K23" s="52">
+      <c r="K23" s="18">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L23" s="53" t="s">
+      <c r="L23" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="M23" s="54">
+      <c r="M23" s="46">
         <v>2.21</v>
       </c>
-      <c r="N23" s="55">
+      <c r="N23" s="47">
         <f t="shared" si="1"/>
         <v>11.05</v>
       </c>
-      <c r="O23" s="55">
+      <c r="O23" s="47">
         <v>2.112</v>
       </c>
-      <c r="P23" s="55">
+      <c r="P23" s="47">
         <f t="shared" si="2"/>
         <v>52.8</v>
       </c>
-      <c r="Q23" s="83"/>
-      <c r="R23" s="85"/>
-      <c r="S23" s="39"/>
-      <c r="T23" s="39"/>
+      <c r="Q23" s="67"/>
+      <c r="R23" s="68"/>
+      <c r="S23" s="34"/>
+      <c r="T23" s="34"/>
     </row>
-    <row r="24" ht="15.75" spans="1:20">
+    <row r="24" customHeight="1" spans="1:20">
       <c r="A24" s="5">
         <f t="shared" si="3"/>
         <v>22</v>
       </c>
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="C24" s="36" t="s">
+      <c r="C24" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="D24" s="37" t="s">
+      <c r="D24" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="E24" s="103" t="s">
-        <v>30</v>
-      </c>
-      <c r="F24" s="103" t="s">
-        <v>30</v>
-      </c>
-      <c r="G24" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="H24" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="I24" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="J24" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="K24" s="103" t="s">
-        <v>30</v>
-      </c>
-      <c r="L24" s="74" t="s">
+      <c r="E24" s="83" t="s">
+        <v>30</v>
+      </c>
+      <c r="F24" s="83" t="s">
+        <v>30</v>
+      </c>
+      <c r="G24" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="H24" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="I24" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="J24" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="K24" s="83" t="s">
+        <v>30</v>
+      </c>
+      <c r="L24" s="48" t="s">
         <v>140</v>
       </c>
-      <c r="M24" s="98" t="s">
-        <v>30</v>
-      </c>
-      <c r="N24" s="103" t="s">
-        <v>30</v>
-      </c>
-      <c r="O24" s="103" t="s">
-        <v>30</v>
-      </c>
-      <c r="P24" s="103" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q24" s="104" t="s">
-        <v>30</v>
-      </c>
-      <c r="R24" s="85"/>
-      <c r="S24" s="39"/>
-      <c r="T24" s="39"/>
+      <c r="M24" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="N24" s="83" t="s">
+        <v>30</v>
+      </c>
+      <c r="O24" s="83" t="s">
+        <v>30</v>
+      </c>
+      <c r="P24" s="83" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q24" s="84" t="s">
+        <v>30</v>
+      </c>
+      <c r="R24" s="68"/>
+      <c r="S24" s="34"/>
+      <c r="T24" s="34"/>
     </row>
-    <row r="25" ht="19.5" spans="1:20">
-      <c r="A25" s="39"/>
-      <c r="B25" s="39"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="39"/>
-      <c r="I25" s="39"/>
-      <c r="J25" s="75" t="s">
+    <row r="25" ht="18" customHeight="1" spans="1:20">
+      <c r="A25" s="34"/>
+      <c r="B25" s="34"/>
+      <c r="C25" t="s">
         <v>141</v>
       </c>
-      <c r="K25" s="75"/>
-      <c r="L25" s="75"/>
-      <c r="M25" s="75"/>
-      <c r="N25" s="76">
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="34"/>
+      <c r="J25" s="59" t="s">
+        <v>142</v>
+      </c>
+      <c r="K25" s="59"/>
+      <c r="L25" s="59"/>
+      <c r="M25" s="59"/>
+      <c r="N25" s="60">
         <f>SUM(N3:N23)</f>
         <v>49.27</v>
       </c>
-      <c r="O25" s="39"/>
-      <c r="P25" s="76">
+      <c r="O25" s="34"/>
+      <c r="P25" s="60">
         <f>SUM(P3:P23)</f>
         <v>233.62</v>
       </c>
-      <c r="Q25" s="91"/>
-      <c r="S25" s="39"/>
-      <c r="T25" s="39"/>
+      <c r="Q25" s="65"/>
+      <c r="S25" s="34"/>
+      <c r="T25" s="34"/>
     </row>
-    <row r="26" ht="18.75" spans="3:16">
-      <c r="C26" t="s">
-        <v>142</v>
-      </c>
-      <c r="J26" s="77" t="s">
+    <row r="26" ht="14" customHeight="1" spans="2:16">
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="K26" s="77"/>
-      <c r="L26" s="77"/>
-      <c r="M26" s="77"/>
-      <c r="P26" s="78">
+      <c r="J26" s="61" t="s">
+        <v>144</v>
+      </c>
+      <c r="K26" s="61"/>
+      <c r="L26" s="61"/>
+      <c r="M26" s="61"/>
+      <c r="P26" s="62">
         <f>P25/5</f>
         <v>46.724</v>
       </c>
     </row>
-    <row r="27" spans="2:3">
-      <c r="B27">
-        <v>1</v>
-      </c>
-      <c r="C27" s="40" t="s">
-        <v>144</v>
+    <row r="27" spans="3:3">
+      <c r="C27" s="36" t="s">
+        <v>91</v>
       </c>
     </row>
-    <row r="28" spans="3:3">
-      <c r="C28" s="41" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="3:3">
-      <c r="C30" s="42"/>
+    <row r="30" hidden="1" spans="3:3">
+      <c r="C30" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3486,7 +3425,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{c209e4de-bf3b-4e84-ab64-8422fab06bbd}</x14:id>
+          <x14:id>{54e1a58a-e616-4df8-abce-d3897a964622}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3500,7 +3439,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{df01a010-2e3f-4c87-b820-10b76fc1ba10}</x14:id>
+          <x14:id>{2a943809-f103-4c74-8138-e2aade31d277}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3526,7 +3465,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{bcaf9097-b6a2-421b-a6a4-7644a1eb9ef0}</x14:id>
+          <x14:id>{969b6976-d947-4cc1-a044-a22e0569acf8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3553,7 +3492,7 @@
     <hyperlink ref="L20" r:id="rId19" display="DIgikey"/>
     <hyperlink ref="L3" r:id="rId20" display="Digikey"/>
     <hyperlink ref="L24" r:id="rId21" display="Aliexpress"/>
-    <hyperlink ref="C28" r:id="rId22" display="Songle relay"/>
+    <hyperlink ref="C27" r:id="rId22" display="Songle relay"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -3561,7 +3500,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{c209e4de-bf3b-4e84-ab64-8422fab06bbd}">
+          <x14:cfRule type="dataBar" id="{54e1a58a-e616-4df8-abce-d3897a964622}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -3574,7 +3513,7 @@
           <xm:sqref>N3:N23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{df01a010-2e3f-4c87-b820-10b76fc1ba10}">
+          <x14:cfRule type="dataBar" id="{2a943809-f103-4c74-8138-e2aade31d277}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -3587,7 +3526,7 @@
           <xm:sqref>P3:P23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{bcaf9097-b6a2-421b-a6a4-7644a1eb9ef0}">
+          <x14:cfRule type="dataBar" id="{969b6976-d947-4cc1-a044-a22e0569acf8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>